<commit_message>
Update schedule UI: show team name instead of draw_code
</commit_message>
<xml_diff>
--- a/App_Complete/DATA.xlsx
+++ b/App_Complete/DATA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APP LONG VIET\XEP LICH THI DAU THE THAO\App_Complete\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A4A3F5E-3259-4795-8C73-C5B68BD22CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7D5E631-1454-4747-A534-37B1355969D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="682" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="682" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BĐ 28.08" sheetId="13" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1648" uniqueCount="871">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1648" uniqueCount="870">
   <si>
     <t>Công ty TNHH Dương Khánh Vinh</t>
   </si>
@@ -2642,6 +2642,9 @@
     <t>Khách mời của TGĐ</t>
   </si>
   <si>
+    <t>TBA</t>
+  </si>
+  <si>
     <t>Nguyễn Huy Quỳnh-Tạ Diệp Anh</t>
   </si>
   <si>
@@ -2709,12 +2712,6 @@
   </si>
   <si>
     <t>Trần Thị Hạnh</t>
-  </si>
-  <si>
-    <t>TBA1</t>
-  </si>
-  <si>
-    <t>TBA2</t>
   </si>
 </sst>
 </file>
@@ -4797,6 +4794,291 @@
     <xf numFmtId="0" fontId="28" fillId="3" borderId="7" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="7" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="24" fillId="8" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="24" fillId="8" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="24" fillId="8" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="7" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4809,308 +5091,23 @@
     <xf numFmtId="20" fontId="7" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="20" fontId="7" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="20" fontId="9" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="20" fontId="7" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="20" fontId="7" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="24" fillId="8" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="24" fillId="8" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="24" fillId="8" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="43" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="45" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="6" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -5560,14 +5557,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" s="18" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="304" t="s">
+      <c r="A1" s="297" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="304"/>
-      <c r="C1" s="304"/>
-      <c r="D1" s="304"/>
-      <c r="E1" s="304"/>
-      <c r="F1" s="304"/>
+      <c r="B1" s="297"/>
+      <c r="C1" s="297"/>
+      <c r="D1" s="297"/>
+      <c r="E1" s="297"/>
+      <c r="F1" s="297"/>
       <c r="G1" s="16"/>
       <c r="H1" s="16"/>
       <c r="I1" s="16"/>
@@ -5585,19 +5582,19 @@
       <c r="U1" s="158"/>
     </row>
     <row r="2" spans="1:21" s="18" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="305" t="s">
+      <c r="A2" s="298" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="305"/>
-      <c r="C2" s="305"/>
-      <c r="D2" s="305"/>
-      <c r="E2" s="305"/>
-      <c r="F2" s="305"/>
-      <c r="G2" s="305"/>
-      <c r="H2" s="305"/>
-      <c r="I2" s="305"/>
-      <c r="J2" s="305"/>
-      <c r="K2" s="305"/>
+      <c r="B2" s="298"/>
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="298"/>
+      <c r="F2" s="298"/>
+      <c r="G2" s="298"/>
+      <c r="H2" s="298"/>
+      <c r="I2" s="298"/>
+      <c r="J2" s="298"/>
+      <c r="K2" s="298"/>
       <c r="L2" s="19"/>
       <c r="M2" s="158"/>
       <c r="N2" s="158"/>
@@ -5696,7 +5693,7 @@
         <v>239</v>
       </c>
       <c r="G5" s="285" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="H5" s="33"/>
       <c r="I5" s="34"/>
@@ -6030,7 +6027,7 @@
         <v>239</v>
       </c>
       <c r="G16" s="287" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="H16" s="71"/>
       <c r="I16" s="61"/>
@@ -6280,7 +6277,7 @@
         <v>241</v>
       </c>
       <c r="G24" s="286" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="H24" s="38"/>
       <c r="I24" s="34"/>
@@ -6841,7 +6838,7 @@
         <v>100</v>
       </c>
       <c r="G41" s="288" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="H41" s="65" t="s">
         <v>803</v>
@@ -6940,7 +6937,7 @@
         <v>100</v>
       </c>
       <c r="G44" s="286" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="H44" s="38"/>
       <c r="I44" s="38"/>
@@ -7126,7 +7123,7 @@
         <v>100</v>
       </c>
       <c r="G50" s="286" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="H50" s="38"/>
       <c r="I50" s="38"/>
@@ -7157,7 +7154,7 @@
         <v>100</v>
       </c>
       <c r="G51" s="286" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="H51" s="38"/>
       <c r="I51" s="38"/>
@@ -7376,7 +7373,7 @@
         <v>1</v>
       </c>
       <c r="G58" s="295" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="H58" s="38"/>
       <c r="I58" s="34"/>
@@ -8338,7 +8335,7 @@
         <v>761</v>
       </c>
       <c r="G89" s="66" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="H89" s="65" t="s">
         <v>803</v>
@@ -8368,7 +8365,7 @@
       <c r="E90" s="37"/>
       <c r="F90" s="38"/>
       <c r="G90" s="38" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="H90" s="38"/>
       <c r="I90" s="47"/>
@@ -8396,7 +8393,7 @@
       <c r="E91" s="37"/>
       <c r="F91" s="38"/>
       <c r="G91" s="38" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="H91" s="50"/>
       <c r="I91" s="47"/>
@@ -8424,7 +8421,7 @@
       <c r="E92" s="37"/>
       <c r="F92" s="38"/>
       <c r="G92" s="38" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="H92" s="50"/>
       <c r="I92" s="47"/>
@@ -8452,7 +8449,7 @@
       <c r="E93" s="37"/>
       <c r="F93" s="38"/>
       <c r="G93" s="38" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="H93" s="50"/>
       <c r="I93" s="47"/>
@@ -8471,7 +8468,7 @@
       <c r="E94" s="37"/>
       <c r="F94" s="38"/>
       <c r="G94" s="38" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="H94" s="38"/>
       <c r="I94" s="47"/>
@@ -8490,7 +8487,7 @@
       <c r="E95" s="37"/>
       <c r="F95" s="38"/>
       <c r="G95" s="38" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="H95" s="38"/>
       <c r="I95" s="47"/>
@@ -8509,7 +8506,7 @@
       <c r="E96" s="37"/>
       <c r="F96" s="38"/>
       <c r="G96" s="38" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="H96" s="38"/>
       <c r="I96" s="47"/>
@@ -8528,7 +8525,7 @@
       <c r="E97" s="37"/>
       <c r="F97" s="38"/>
       <c r="G97" s="38" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="H97" s="38"/>
       <c r="I97" s="47"/>
@@ -8547,7 +8544,7 @@
       <c r="E98" s="37"/>
       <c r="F98" s="38"/>
       <c r="G98" s="38" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="H98" s="38"/>
       <c r="I98" s="47"/>
@@ -8566,7 +8563,7 @@
       <c r="E99" s="70"/>
       <c r="F99" s="71"/>
       <c r="G99" s="71" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="H99" s="71"/>
       <c r="I99" s="164"/>
@@ -8585,7 +8582,7 @@
       <c r="E100" s="54"/>
       <c r="F100" s="55"/>
       <c r="G100" s="55" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="H100" s="55"/>
       <c r="I100" s="56"/>
@@ -8643,14 +8640,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="112" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="306" t="s">
+      <c r="A1" s="299" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="306"/>
-      <c r="C1" s="306"/>
-      <c r="D1" s="306"/>
-      <c r="E1" s="306"/>
-      <c r="F1" s="306"/>
+      <c r="B1" s="299"/>
+      <c r="C1" s="299"/>
+      <c r="D1" s="299"/>
+      <c r="E1" s="299"/>
+      <c r="F1" s="299"/>
       <c r="G1" s="110"/>
       <c r="H1" s="110"/>
       <c r="I1" s="110"/>
@@ -8660,20 +8657,20 @@
       <c r="M1" s="111"/>
     </row>
     <row r="2" spans="1:14" s="112" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="307" t="s">
+      <c r="A2" s="300" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="307"/>
-      <c r="C2" s="307"/>
-      <c r="D2" s="307"/>
-      <c r="E2" s="307"/>
-      <c r="F2" s="307"/>
-      <c r="G2" s="307"/>
-      <c r="H2" s="307"/>
-      <c r="I2" s="307"/>
-      <c r="J2" s="307"/>
-      <c r="K2" s="307"/>
-      <c r="L2" s="307"/>
+      <c r="B2" s="300"/>
+      <c r="C2" s="300"/>
+      <c r="D2" s="300"/>
+      <c r="E2" s="300"/>
+      <c r="F2" s="300"/>
+      <c r="G2" s="300"/>
+      <c r="H2" s="300"/>
+      <c r="I2" s="300"/>
+      <c r="J2" s="300"/>
+      <c r="K2" s="300"/>
+      <c r="L2" s="300"/>
       <c r="M2" s="113"/>
       <c r="N2" s="113"/>
     </row>
@@ -10511,16 +10508,16 @@
         <v>845</v>
       </c>
       <c r="G60" s="268" t="s">
-        <v>869</v>
+        <v>846</v>
       </c>
       <c r="H60" s="268" t="s">
-        <v>870</v>
+        <v>846</v>
       </c>
       <c r="I60" s="137"/>
       <c r="J60" s="137"/>
       <c r="K60" s="137"/>
       <c r="L60" s="282" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
     </row>
     <row r="61" spans="1:12" s="126" customFormat="1" x14ac:dyDescent="0.25">
@@ -10855,7 +10852,7 @@
         <v>799</v>
       </c>
       <c r="H71" s="284" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="I71" s="151"/>
       <c r="J71" s="151"/>
@@ -10886,7 +10883,7 @@
         <v>343</v>
       </c>
       <c r="H72" s="296" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="I72" s="151"/>
       <c r="J72" s="151"/>
@@ -11120,10 +11117,10 @@
       <c r="G2" s="198" t="s">
         <v>220</v>
       </c>
-      <c r="H2" s="308" t="s">
+      <c r="H2" s="310" t="s">
         <v>228</v>
       </c>
-      <c r="I2" s="309" t="s">
+      <c r="I2" s="303" t="s">
         <v>232</v>
       </c>
     </row>
@@ -11134,27 +11131,27 @@
       <c r="G3" s="198" t="s">
         <v>221</v>
       </c>
-      <c r="H3" s="308"/>
-      <c r="I3" s="309"/>
+      <c r="H3" s="310"/>
+      <c r="I3" s="303"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="311" t="s">
+      <c r="A4" s="302" t="s">
         <v>350</v>
       </c>
-      <c r="B4" s="311"/>
-      <c r="C4" s="311"/>
-      <c r="D4" s="311"/>
+      <c r="B4" s="302"/>
+      <c r="C4" s="302"/>
+      <c r="D4" s="302"/>
       <c r="E4" s="255"/>
       <c r="F4" s="255"/>
-      <c r="I4" s="309"/>
+      <c r="I4" s="303"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="309" t="s">
+      <c r="A5" s="303" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="309"/>
-      <c r="C5" s="309"/>
-      <c r="D5" s="309"/>
+      <c r="B5" s="303"/>
+      <c r="C5" s="303"/>
+      <c r="D5" s="303"/>
       <c r="E5" s="256"/>
       <c r="F5" s="256" t="s">
         <v>341</v>
@@ -11162,18 +11159,18 @@
       <c r="G5" s="198" t="s">
         <v>222</v>
       </c>
-      <c r="H5" s="308" t="s">
+      <c r="H5" s="310" t="s">
         <v>229</v>
       </c>
-      <c r="I5" s="309"/>
+      <c r="I5" s="303"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="309" t="s">
+      <c r="A6" s="303" t="s">
         <v>352</v>
       </c>
-      <c r="B6" s="309"/>
-      <c r="C6" s="309"/>
-      <c r="D6" s="309"/>
+      <c r="B6" s="303"/>
+      <c r="C6" s="303"/>
+      <c r="D6" s="303"/>
       <c r="E6" s="256"/>
       <c r="F6" s="256" t="s">
         <v>234</v>
@@ -11181,8 +11178,8 @@
       <c r="G6" s="198" t="s">
         <v>223</v>
       </c>
-      <c r="H6" s="308"/>
-      <c r="I6" s="309"/>
+      <c r="H6" s="310"/>
+      <c r="I6" s="303"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="199" t="s">
@@ -11194,10 +11191,10 @@
       <c r="G8" s="198" t="s">
         <v>224</v>
       </c>
-      <c r="H8" s="308" t="s">
+      <c r="H8" s="310" t="s">
         <v>230</v>
       </c>
-      <c r="I8" s="309" t="s">
+      <c r="I8" s="303" t="s">
         <v>233</v>
       </c>
     </row>
@@ -11208,8 +11205,8 @@
       <c r="G9" s="198" t="s">
         <v>225</v>
       </c>
-      <c r="H9" s="308"/>
-      <c r="I9" s="309"/>
+      <c r="H9" s="310"/>
+      <c r="I9" s="303"/>
     </row>
     <row r="10" spans="1:9" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="200" t="s">
@@ -11226,7 +11223,7 @@
       </c>
       <c r="E10" s="255"/>
       <c r="F10" s="255"/>
-      <c r="I10" s="309"/>
+      <c r="I10" s="303"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="203">
@@ -11246,10 +11243,10 @@
       <c r="G11" s="198" t="s">
         <v>226</v>
       </c>
-      <c r="H11" s="308" t="s">
+      <c r="H11" s="310" t="s">
         <v>231</v>
       </c>
-      <c r="I11" s="309"/>
+      <c r="I11" s="303"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
@@ -11268,8 +11265,8 @@
       <c r="G12" s="198" t="s">
         <v>227</v>
       </c>
-      <c r="H12" s="308"/>
-      <c r="I12" s="309"/>
+      <c r="H12" s="310"/>
+      <c r="I12" s="303"/>
     </row>
     <row r="13" spans="1:9" s="209" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7">
@@ -11342,26 +11339,26 @@
       <c r="A22" s="2"/>
     </row>
     <row r="23" spans="1:6" s="209" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="317" t="s">
+      <c r="A23" s="309" t="s">
         <v>3</v>
       </c>
       <c r="B23" s="198" t="s">
         <v>316</v>
       </c>
-      <c r="C23" s="312" t="s">
+      <c r="C23" s="304" t="s">
         <v>15</v>
       </c>
-      <c r="D23" s="315"/>
+      <c r="D23" s="307"/>
       <c r="E23" s="255"/>
       <c r="F23" s="255"/>
     </row>
     <row r="24" spans="1:6" ht="41.4" x14ac:dyDescent="0.25">
-      <c r="A24" s="317"/>
+      <c r="A24" s="309"/>
       <c r="B24" s="214" t="s">
         <v>357</v>
       </c>
-      <c r="C24" s="314"/>
-      <c r="D24" s="316"/>
+      <c r="C24" s="306"/>
+      <c r="D24" s="308"/>
       <c r="E24" s="255"/>
       <c r="F24" s="255"/>
     </row>
@@ -11371,38 +11368,38 @@
       </c>
     </row>
     <row r="28" spans="1:6" s="209" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="317" t="s">
+      <c r="A28" s="309" t="s">
         <v>4</v>
       </c>
       <c r="B28" s="198" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="312" t="s">
+      <c r="C28" s="304" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="315"/>
+      <c r="D28" s="307"/>
       <c r="E28" s="255"/>
-      <c r="F28" s="310"/>
+      <c r="F28" s="301"/>
     </row>
     <row r="29" spans="1:6" s="209" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="317"/>
+      <c r="A29" s="309"/>
       <c r="B29" s="198" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="313"/>
-      <c r="D29" s="316"/>
+      <c r="C29" s="305"/>
+      <c r="D29" s="308"/>
       <c r="E29" s="255"/>
-      <c r="F29" s="310"/>
+      <c r="F29" s="301"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="317"/>
+      <c r="A30" s="309"/>
       <c r="B30" s="198" t="s">
         <v>19</v>
       </c>
-      <c r="C30" s="314"/>
-      <c r="D30" s="316"/>
+      <c r="C30" s="306"/>
+      <c r="D30" s="308"/>
       <c r="E30" s="255"/>
-      <c r="F30" s="310"/>
+      <c r="F30" s="301"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
@@ -11481,6 +11478,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I2:I6"/>
+    <mergeCell ref="I8:I12"/>
     <mergeCell ref="F28:F30"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A5:D5"/>
@@ -11491,12 +11494,6 @@
     <mergeCell ref="A28:A30"/>
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="C23:C24"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I2:I6"/>
-    <mergeCell ref="I8:I12"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -11534,29 +11531,29 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="311" t="s">
+      <c r="A4" s="302" t="s">
         <v>351</v>
       </c>
-      <c r="B4" s="311"/>
-      <c r="C4" s="311"/>
-      <c r="D4" s="311"/>
+      <c r="B4" s="302"/>
+      <c r="C4" s="302"/>
+      <c r="D4" s="302"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="309" t="str">
+      <c r="A5" s="303" t="str">
         <f>'[1]BĐ Nam'!A5:D5</f>
         <v>Địa điểm: Khu liên hiệp thể thao Thanh Hà - Hà Nội</v>
       </c>
-      <c r="B5" s="309"/>
-      <c r="C5" s="309"/>
-      <c r="D5" s="309"/>
+      <c r="B5" s="303"/>
+      <c r="C5" s="303"/>
+      <c r="D5" s="303"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="309" t="s">
+      <c r="A6" s="303" t="s">
         <v>352</v>
       </c>
-      <c r="B6" s="309"/>
-      <c r="C6" s="309"/>
-      <c r="D6" s="309"/>
+      <c r="B6" s="303"/>
+      <c r="C6" s="303"/>
+      <c r="D6" s="303"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="199" t="s">
@@ -11870,13 +11867,13 @@
       <c r="I41" s="209"/>
     </row>
     <row r="42" spans="1:9" s="209" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="321" t="s">
+      <c r="A42" s="314" t="s">
         <v>3</v>
       </c>
       <c r="B42" s="214" t="s">
         <v>321</v>
       </c>
-      <c r="C42" s="312" t="s">
+      <c r="C42" s="304" t="s">
         <v>387</v>
       </c>
       <c r="D42" s="2"/>
@@ -11885,11 +11882,11 @@
       <c r="G42" s="255"/>
     </row>
     <row r="43" spans="1:9" s="209" customFormat="1" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A43" s="322"/>
+      <c r="A43" s="315"/>
       <c r="B43" s="214" t="s">
         <v>322</v>
       </c>
-      <c r="C43" s="314"/>
+      <c r="C43" s="306"/>
       <c r="D43" s="2"/>
       <c r="E43" s="255"/>
       <c r="F43" s="255"/>
@@ -11905,29 +11902,29 @@
       </c>
     </row>
     <row r="47" spans="1:9" s="209" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="317" t="s">
+      <c r="A47" s="309" t="s">
         <v>4</v>
       </c>
-      <c r="B47" s="318" t="s">
+      <c r="B47" s="311" t="s">
         <v>323</v>
       </c>
-      <c r="C47" s="312" t="s">
+      <c r="C47" s="304" t="s">
         <v>325</v>
       </c>
       <c r="D47" s="275"/>
       <c r="E47" s="256"/>
     </row>
     <row r="48" spans="1:9" s="209" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="317"/>
-      <c r="B48" s="319"/>
-      <c r="C48" s="313"/>
+      <c r="A48" s="309"/>
+      <c r="B48" s="312"/>
+      <c r="C48" s="305"/>
       <c r="D48" s="275"/>
       <c r="E48" s="256"/>
     </row>
     <row r="49" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="317"/>
-      <c r="B49" s="320"/>
-      <c r="C49" s="314"/>
+      <c r="A49" s="309"/>
+      <c r="B49" s="313"/>
+      <c r="C49" s="306"/>
       <c r="D49" s="275"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -12131,70 +12128,70 @@
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="311" t="s">
+      <c r="A3" s="302" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="311"/>
-      <c r="C3" s="311"/>
-      <c r="D3" s="311"/>
-      <c r="E3" s="311"/>
-      <c r="F3" s="311"/>
-      <c r="G3" s="311"/>
-      <c r="H3" s="311"/>
-      <c r="I3" s="311"/>
-      <c r="J3" s="311"/>
-      <c r="K3" s="311"/>
-      <c r="L3" s="311"/>
-      <c r="M3" s="311"/>
-      <c r="N3" s="311"/>
-      <c r="O3" s="311"/>
-      <c r="P3" s="311"/>
+      <c r="B3" s="302"/>
+      <c r="C3" s="302"/>
+      <c r="D3" s="302"/>
+      <c r="E3" s="302"/>
+      <c r="F3" s="302"/>
+      <c r="G3" s="302"/>
+      <c r="H3" s="302"/>
+      <c r="I3" s="302"/>
+      <c r="J3" s="302"/>
+      <c r="K3" s="302"/>
+      <c r="L3" s="302"/>
+      <c r="M3" s="302"/>
+      <c r="N3" s="302"/>
+      <c r="O3" s="302"/>
+      <c r="P3" s="302"/>
       <c r="R3" s="2" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" s="309" t="s">
+      <c r="A4" s="303" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="309"/>
-      <c r="C4" s="309"/>
-      <c r="D4" s="309"/>
-      <c r="E4" s="309"/>
-      <c r="F4" s="309"/>
-      <c r="G4" s="309"/>
-      <c r="H4" s="309"/>
-      <c r="I4" s="309"/>
-      <c r="J4" s="309"/>
-      <c r="K4" s="309"/>
-      <c r="L4" s="309"/>
-      <c r="M4" s="309"/>
-      <c r="N4" s="309"/>
-      <c r="O4" s="309"/>
-      <c r="P4" s="309"/>
+      <c r="B4" s="303"/>
+      <c r="C4" s="303"/>
+      <c r="D4" s="303"/>
+      <c r="E4" s="303"/>
+      <c r="F4" s="303"/>
+      <c r="G4" s="303"/>
+      <c r="H4" s="303"/>
+      <c r="I4" s="303"/>
+      <c r="J4" s="303"/>
+      <c r="K4" s="303"/>
+      <c r="L4" s="303"/>
+      <c r="M4" s="303"/>
+      <c r="N4" s="303"/>
+      <c r="O4" s="303"/>
+      <c r="P4" s="303"/>
       <c r="R4" s="2" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" s="309" t="s">
+      <c r="A5" s="303" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="309"/>
-      <c r="C5" s="309"/>
-      <c r="D5" s="309"/>
-      <c r="E5" s="309"/>
-      <c r="F5" s="309"/>
-      <c r="G5" s="309"/>
-      <c r="H5" s="309"/>
-      <c r="I5" s="309"/>
-      <c r="J5" s="309"/>
-      <c r="K5" s="309"/>
-      <c r="L5" s="309"/>
-      <c r="M5" s="309"/>
-      <c r="N5" s="309"/>
-      <c r="O5" s="309"/>
-      <c r="P5" s="309"/>
+      <c r="B5" s="303"/>
+      <c r="C5" s="303"/>
+      <c r="D5" s="303"/>
+      <c r="E5" s="303"/>
+      <c r="F5" s="303"/>
+      <c r="G5" s="303"/>
+      <c r="H5" s="303"/>
+      <c r="I5" s="303"/>
+      <c r="J5" s="303"/>
+      <c r="K5" s="303"/>
+      <c r="L5" s="303"/>
+      <c r="M5" s="303"/>
+      <c r="N5" s="303"/>
+      <c r="O5" s="303"/>
+      <c r="P5" s="303"/>
       <c r="R5" s="2" t="s">
         <v>267</v>
       </c>
@@ -12211,36 +12208,36 @@
       </c>
     </row>
     <row r="7" spans="1:19" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="326" t="s">
+      <c r="A7" s="344" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="329" t="s">
+      <c r="B7" s="347" t="s">
         <v>270</v>
       </c>
-      <c r="C7" s="329" t="s">
+      <c r="C7" s="347" t="s">
         <v>271</v>
       </c>
-      <c r="D7" s="329" t="s">
+      <c r="D7" s="347" t="s">
         <v>269</v>
       </c>
-      <c r="E7" s="323" t="s">
+      <c r="E7" s="341" t="s">
         <v>268</v>
       </c>
-      <c r="F7" s="324"/>
-      <c r="G7" s="324"/>
-      <c r="H7" s="324"/>
-      <c r="I7" s="324"/>
-      <c r="J7" s="324"/>
-      <c r="K7" s="324"/>
-      <c r="L7" s="324"/>
-      <c r="M7" s="332"/>
-      <c r="N7" s="333" t="s">
+      <c r="F7" s="342"/>
+      <c r="G7" s="342"/>
+      <c r="H7" s="342"/>
+      <c r="I7" s="342"/>
+      <c r="J7" s="342"/>
+      <c r="K7" s="342"/>
+      <c r="L7" s="342"/>
+      <c r="M7" s="350"/>
+      <c r="N7" s="351" t="s">
         <v>41</v>
       </c>
-      <c r="O7" s="335" t="s">
+      <c r="O7" s="353" t="s">
         <v>10</v>
       </c>
-      <c r="P7" s="336"/>
+      <c r="P7" s="354"/>
       <c r="R7" s="2">
         <v>24</v>
       </c>
@@ -12249,26 +12246,26 @@
       </c>
     </row>
     <row r="8" spans="1:19" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="327"/>
-      <c r="B8" s="330"/>
-      <c r="C8" s="330"/>
-      <c r="D8" s="330"/>
-      <c r="E8" s="323" t="s">
+      <c r="A8" s="345"/>
+      <c r="B8" s="348"/>
+      <c r="C8" s="348"/>
+      <c r="D8" s="348"/>
+      <c r="E8" s="341" t="s">
         <v>774</v>
       </c>
-      <c r="F8" s="324"/>
-      <c r="G8" s="324"/>
-      <c r="H8" s="324"/>
-      <c r="I8" s="324"/>
-      <c r="J8" s="324"/>
-      <c r="K8" s="325"/>
-      <c r="L8" s="340" t="s">
+      <c r="F8" s="342"/>
+      <c r="G8" s="342"/>
+      <c r="H8" s="342"/>
+      <c r="I8" s="342"/>
+      <c r="J8" s="342"/>
+      <c r="K8" s="343"/>
+      <c r="L8" s="358" t="s">
         <v>276</v>
       </c>
-      <c r="M8" s="332"/>
-      <c r="N8" s="334"/>
-      <c r="O8" s="316"/>
-      <c r="P8" s="337"/>
+      <c r="M8" s="350"/>
+      <c r="N8" s="352"/>
+      <c r="O8" s="308"/>
+      <c r="P8" s="355"/>
       <c r="R8" s="2">
         <v>16</v>
       </c>
@@ -12277,10 +12274,10 @@
       </c>
     </row>
     <row r="9" spans="1:19" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="328"/>
-      <c r="B9" s="331"/>
-      <c r="C9" s="331"/>
-      <c r="D9" s="331"/>
+      <c r="A9" s="346"/>
+      <c r="B9" s="349"/>
+      <c r="C9" s="349"/>
+      <c r="D9" s="349"/>
       <c r="E9" s="257" t="s">
         <v>277</v>
       </c>
@@ -12308,9 +12305,9 @@
       <c r="M9" s="257" t="s">
         <v>278</v>
       </c>
-      <c r="N9" s="331"/>
-      <c r="O9" s="338"/>
-      <c r="P9" s="339"/>
+      <c r="N9" s="349"/>
+      <c r="O9" s="356"/>
+      <c r="P9" s="357"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
@@ -12352,228 +12349,228 @@
         <f>C11-B11</f>
         <v>2.083333333333337E-2</v>
       </c>
-      <c r="E11" s="344" t="s">
+      <c r="E11" s="318" t="s">
         <v>272</v>
       </c>
-      <c r="F11" s="345"/>
-      <c r="G11" s="345"/>
-      <c r="H11" s="345"/>
-      <c r="I11" s="345"/>
-      <c r="J11" s="345"/>
-      <c r="K11" s="345"/>
-      <c r="L11" s="345"/>
-      <c r="M11" s="346"/>
+      <c r="F11" s="319"/>
+      <c r="G11" s="319"/>
+      <c r="H11" s="319"/>
+      <c r="I11" s="319"/>
+      <c r="J11" s="319"/>
+      <c r="K11" s="319"/>
+      <c r="L11" s="319"/>
+      <c r="M11" s="320"/>
       <c r="N11" s="9" t="s">
         <v>284</v>
       </c>
       <c r="O11" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="P11" s="341" t="s">
+      <c r="P11" s="324" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="12" spans="1:19" s="274" customFormat="1" ht="49.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="297">
+      <c r="A12" s="392">
         <f>A11+1</f>
         <v>2</v>
       </c>
-      <c r="B12" s="298">
+      <c r="B12" s="393">
         <f t="shared" ref="B12" si="0">C11</f>
         <v>0.35416666666666669</v>
       </c>
-      <c r="C12" s="298">
+      <c r="C12" s="393">
         <v>0.36458333333333331</v>
       </c>
-      <c r="D12" s="298">
+      <c r="D12" s="393">
         <f>C12-B12</f>
         <v>1.041666666666663E-2</v>
       </c>
-      <c r="E12" s="299" t="s">
+      <c r="E12" s="394" t="s">
         <v>399</v>
       </c>
-      <c r="F12" s="299" t="s">
+      <c r="F12" s="394" t="s">
         <v>400</v>
       </c>
-      <c r="G12" s="299" t="s">
+      <c r="G12" s="394" t="s">
         <v>401</v>
       </c>
-      <c r="H12" s="299" t="s">
+      <c r="H12" s="394" t="s">
         <v>402</v>
       </c>
-      <c r="I12" s="299" t="s">
+      <c r="I12" s="394" t="s">
         <v>403</v>
       </c>
-      <c r="J12" s="300" t="s">
+      <c r="J12" s="395" t="s">
         <v>399</v>
       </c>
-      <c r="K12" s="300" t="s">
+      <c r="K12" s="395" t="s">
         <v>400</v>
       </c>
-      <c r="L12" s="361" t="s">
+      <c r="L12" s="396" t="s">
         <v>279</v>
       </c>
-      <c r="M12" s="361" t="s">
+      <c r="M12" s="396" t="s">
         <v>280</v>
       </c>
       <c r="N12" s="10" t="s">
         <v>608</v>
       </c>
-      <c r="O12" s="347" t="s">
+      <c r="O12" s="327" t="s">
         <v>297</v>
       </c>
-      <c r="P12" s="342"/>
+      <c r="P12" s="325"/>
     </row>
     <row r="13" spans="1:19" s="274" customFormat="1" ht="49.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="297">
+      <c r="A13" s="392">
         <f t="shared" ref="A13:A35" si="1">A12+1</f>
         <v>3</v>
       </c>
-      <c r="B13" s="298">
+      <c r="B13" s="393">
         <f>C12</f>
         <v>0.36458333333333331</v>
       </c>
-      <c r="C13" s="298">
+      <c r="C13" s="393">
         <v>0.375</v>
       </c>
-      <c r="D13" s="298">
+      <c r="D13" s="393">
         <f t="shared" ref="D13:D35" si="2">C13-B13</f>
         <v>1.0416666666666685E-2</v>
       </c>
-      <c r="E13" s="299" t="s">
+      <c r="E13" s="394" t="s">
         <v>404</v>
       </c>
-      <c r="F13" s="299" t="s">
+      <c r="F13" s="394" t="s">
         <v>405</v>
       </c>
-      <c r="G13" s="299" t="s">
+      <c r="G13" s="394" t="s">
         <v>406</v>
       </c>
-      <c r="H13" s="299" t="s">
+      <c r="H13" s="394" t="s">
         <v>407</v>
       </c>
-      <c r="I13" s="299" t="s">
+      <c r="I13" s="394" t="s">
         <v>408</v>
       </c>
-      <c r="J13" s="300" t="s">
+      <c r="J13" s="395" t="s">
         <v>401</v>
       </c>
-      <c r="K13" s="300" t="s">
+      <c r="K13" s="395" t="s">
         <v>402</v>
       </c>
-      <c r="L13" s="362"/>
-      <c r="M13" s="362"/>
+      <c r="L13" s="397"/>
+      <c r="M13" s="397"/>
       <c r="N13" s="10"/>
-      <c r="O13" s="348"/>
-      <c r="P13" s="342"/>
+      <c r="O13" s="328"/>
+      <c r="P13" s="325"/>
     </row>
     <row r="14" spans="1:19" s="274" customFormat="1" ht="49.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="297">
+      <c r="A14" s="392">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="B14" s="298">
+      <c r="B14" s="393">
         <f>C13</f>
         <v>0.375</v>
       </c>
-      <c r="C14" s="298">
+      <c r="C14" s="393">
         <v>0.38541666666666669</v>
       </c>
-      <c r="D14" s="298">
+      <c r="D14" s="393">
         <f t="shared" si="2"/>
         <v>1.0416666666666685E-2</v>
       </c>
-      <c r="E14" s="299" t="s">
+      <c r="E14" s="394" t="s">
         <v>409</v>
       </c>
-      <c r="F14" s="299" t="s">
+      <c r="F14" s="394" t="s">
         <v>410</v>
       </c>
-      <c r="G14" s="299" t="s">
+      <c r="G14" s="394" t="s">
         <v>411</v>
       </c>
-      <c r="H14" s="299" t="s">
+      <c r="H14" s="394" t="s">
         <v>412</v>
       </c>
-      <c r="I14" s="299" t="s">
+      <c r="I14" s="394" t="s">
         <v>413</v>
       </c>
-      <c r="J14" s="300" t="s">
+      <c r="J14" s="395" t="s">
         <v>403</v>
       </c>
-      <c r="K14" s="300" t="s">
+      <c r="K14" s="395" t="s">
         <v>404</v>
       </c>
-      <c r="L14" s="362"/>
-      <c r="M14" s="362"/>
+      <c r="L14" s="397"/>
+      <c r="M14" s="397"/>
       <c r="N14" s="10"/>
-      <c r="O14" s="348"/>
-      <c r="P14" s="342"/>
+      <c r="O14" s="328"/>
+      <c r="P14" s="325"/>
     </row>
     <row r="15" spans="1:19" s="274" customFormat="1" ht="49.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="297">
+      <c r="A15" s="392">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="B15" s="298">
+      <c r="B15" s="393">
         <f>C14</f>
         <v>0.38541666666666669</v>
       </c>
-      <c r="C15" s="298">
+      <c r="C15" s="393">
         <v>0.39583333333333331</v>
       </c>
-      <c r="D15" s="298">
+      <c r="D15" s="393">
         <f t="shared" si="2"/>
         <v>1.041666666666663E-2</v>
       </c>
-      <c r="E15" s="301" t="s">
+      <c r="E15" s="398" t="s">
         <v>449</v>
       </c>
-      <c r="F15" s="301" t="s">
+      <c r="F15" s="398" t="s">
         <v>457</v>
       </c>
-      <c r="G15" s="301" t="s">
+      <c r="G15" s="398" t="s">
         <v>450</v>
       </c>
-      <c r="H15" s="301" t="s">
+      <c r="H15" s="398" t="s">
         <v>458</v>
       </c>
-      <c r="I15" s="299" t="s">
+      <c r="I15" s="394" t="s">
         <v>414</v>
       </c>
-      <c r="J15" s="300" t="s">
+      <c r="J15" s="395" t="s">
         <v>405</v>
       </c>
-      <c r="K15" s="300" t="s">
+      <c r="K15" s="395" t="s">
         <v>406</v>
       </c>
-      <c r="L15" s="363"/>
-      <c r="M15" s="363"/>
+      <c r="L15" s="399"/>
+      <c r="M15" s="399"/>
       <c r="N15" s="244" t="s">
         <v>609</v>
       </c>
-      <c r="O15" s="348"/>
-      <c r="P15" s="342"/>
+      <c r="O15" s="328"/>
+      <c r="P15" s="325"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
-      <c r="E16" s="344" t="s">
+      <c r="E16" s="318" t="s">
         <v>612</v>
       </c>
-      <c r="F16" s="345"/>
-      <c r="G16" s="345"/>
-      <c r="H16" s="345"/>
-      <c r="I16" s="345"/>
-      <c r="J16" s="345"/>
-      <c r="K16" s="345"/>
-      <c r="L16" s="345"/>
-      <c r="M16" s="346"/>
+      <c r="F16" s="319"/>
+      <c r="G16" s="319"/>
+      <c r="H16" s="319"/>
+      <c r="I16" s="319"/>
+      <c r="J16" s="319"/>
+      <c r="K16" s="319"/>
+      <c r="L16" s="319"/>
+      <c r="M16" s="320"/>
       <c r="N16" s="10"/>
-      <c r="O16" s="348"/>
-      <c r="P16" s="342"/>
+      <c r="O16" s="328"/>
+      <c r="P16" s="325"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
@@ -12612,15 +12609,15 @@
       <c r="K17" s="245" t="s">
         <v>453</v>
       </c>
-      <c r="L17" s="352" t="s">
+      <c r="L17" s="316" t="s">
         <v>281</v>
       </c>
-      <c r="M17" s="352" t="s">
+      <c r="M17" s="316" t="s">
         <v>282</v>
       </c>
       <c r="N17" s="10"/>
-      <c r="O17" s="348"/>
-      <c r="P17" s="342"/>
+      <c r="O17" s="328"/>
+      <c r="P17" s="325"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="7">
@@ -12659,11 +12656,11 @@
       <c r="K18" s="245" t="s">
         <v>454</v>
       </c>
-      <c r="L18" s="353"/>
-      <c r="M18" s="353"/>
+      <c r="L18" s="317"/>
+      <c r="M18" s="317"/>
       <c r="N18" s="10"/>
-      <c r="O18" s="348"/>
-      <c r="P18" s="342"/>
+      <c r="O18" s="328"/>
+      <c r="P18" s="325"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="7">
@@ -12702,13 +12699,13 @@
       <c r="K19" s="245" t="s">
         <v>455</v>
       </c>
-      <c r="L19" s="353"/>
-      <c r="M19" s="353"/>
+      <c r="L19" s="317"/>
+      <c r="M19" s="317"/>
       <c r="N19" s="10" t="s">
         <v>610</v>
       </c>
-      <c r="O19" s="348"/>
-      <c r="P19" s="342"/>
+      <c r="O19" s="328"/>
+      <c r="P19" s="325"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="7">
@@ -12747,31 +12744,31 @@
       <c r="K20" s="106" t="s">
         <v>530</v>
       </c>
-      <c r="L20" s="364"/>
-      <c r="M20" s="364"/>
+      <c r="L20" s="339"/>
+      <c r="M20" s="339"/>
       <c r="N20" s="10"/>
-      <c r="O20" s="348"/>
-      <c r="P20" s="342"/>
+      <c r="O20" s="328"/>
+      <c r="P20" s="325"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
       <c r="D21" s="8"/>
-      <c r="E21" s="344" t="s">
+      <c r="E21" s="318" t="s">
         <v>613</v>
       </c>
-      <c r="F21" s="345"/>
-      <c r="G21" s="345"/>
-      <c r="H21" s="345"/>
-      <c r="I21" s="345"/>
-      <c r="J21" s="345"/>
-      <c r="K21" s="345"/>
-      <c r="L21" s="345"/>
-      <c r="M21" s="346"/>
+      <c r="F21" s="319"/>
+      <c r="G21" s="319"/>
+      <c r="H21" s="319"/>
+      <c r="I21" s="319"/>
+      <c r="J21" s="319"/>
+      <c r="K21" s="319"/>
+      <c r="L21" s="319"/>
+      <c r="M21" s="320"/>
       <c r="N21" s="10"/>
-      <c r="O21" s="348"/>
-      <c r="P21" s="342"/>
+      <c r="O21" s="328"/>
+      <c r="P21" s="325"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
@@ -12815,8 +12812,8 @@
       <c r="N22" s="244" t="s">
         <v>611</v>
       </c>
-      <c r="O22" s="348"/>
-      <c r="P22" s="342"/>
+      <c r="O22" s="328"/>
+      <c r="P22" s="325"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="7">
@@ -12854,8 +12851,8 @@
       <c r="L23" s="8"/>
       <c r="M23" s="8"/>
       <c r="N23" s="9"/>
-      <c r="O23" s="348"/>
-      <c r="P23" s="342"/>
+      <c r="O23" s="328"/>
+      <c r="P23" s="325"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
@@ -12873,32 +12870,32 @@
         <f t="shared" si="2"/>
         <v>1.0416666666666685E-2</v>
       </c>
-      <c r="E24" s="302" t="s">
+      <c r="E24" s="400" t="s">
         <v>648</v>
       </c>
-      <c r="F24" s="302" t="s">
+      <c r="F24" s="400" t="s">
         <v>651</v>
       </c>
-      <c r="G24" s="302" t="s">
+      <c r="G24" s="400" t="s">
         <v>654</v>
       </c>
-      <c r="H24" s="302" t="s">
+      <c r="H24" s="400" t="s">
         <v>657</v>
       </c>
-      <c r="I24" s="302" t="s">
+      <c r="I24" s="400" t="s">
         <v>660</v>
       </c>
-      <c r="J24" s="302" t="s">
+      <c r="J24" s="400" t="s">
         <v>663</v>
       </c>
-      <c r="K24" s="302" t="s">
+      <c r="K24" s="400" t="s">
         <v>666</v>
       </c>
       <c r="L24" s="8"/>
       <c r="M24" s="8"/>
       <c r="N24" s="9"/>
-      <c r="O24" s="349"/>
-      <c r="P24" s="342"/>
+      <c r="O24" s="329"/>
+      <c r="P24" s="325"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="7">
@@ -12916,32 +12913,32 @@
         <f t="shared" si="2"/>
         <v>1.0416666666666685E-2</v>
       </c>
-      <c r="E25" s="302" t="s">
+      <c r="E25" s="400" t="s">
         <v>649</v>
       </c>
-      <c r="F25" s="302" t="s">
+      <c r="F25" s="400" t="s">
         <v>652</v>
       </c>
-      <c r="G25" s="302" t="s">
+      <c r="G25" s="400" t="s">
         <v>655</v>
       </c>
-      <c r="H25" s="302" t="s">
+      <c r="H25" s="400" t="s">
         <v>658</v>
       </c>
-      <c r="I25" s="302" t="s">
+      <c r="I25" s="400" t="s">
         <v>661</v>
       </c>
-      <c r="J25" s="302" t="s">
+      <c r="J25" s="400" t="s">
         <v>664</v>
       </c>
-      <c r="K25" s="302" t="s">
+      <c r="K25" s="400" t="s">
         <v>669</v>
       </c>
       <c r="L25" s="8"/>
       <c r="M25" s="8"/>
       <c r="N25" s="9"/>
       <c r="O25" s="242"/>
-      <c r="P25" s="342"/>
+      <c r="P25" s="325"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
@@ -12959,32 +12956,32 @@
         <f t="shared" si="2"/>
         <v>1.041666666666663E-2</v>
       </c>
-      <c r="E26" s="302" t="s">
+      <c r="E26" s="400" t="s">
         <v>650</v>
       </c>
-      <c r="F26" s="302" t="s">
+      <c r="F26" s="400" t="s">
         <v>653</v>
       </c>
-      <c r="G26" s="302" t="s">
+      <c r="G26" s="400" t="s">
         <v>656</v>
       </c>
-      <c r="H26" s="302" t="s">
+      <c r="H26" s="400" t="s">
         <v>659</v>
       </c>
-      <c r="I26" s="302" t="s">
+      <c r="I26" s="400" t="s">
         <v>662</v>
       </c>
-      <c r="J26" s="302" t="s">
+      <c r="J26" s="400" t="s">
         <v>667</v>
       </c>
-      <c r="K26" s="302" t="s">
+      <c r="K26" s="400" t="s">
         <v>670</v>
       </c>
       <c r="L26" s="8"/>
       <c r="M26" s="8"/>
       <c r="N26" s="9"/>
       <c r="O26" s="242"/>
-      <c r="P26" s="342"/>
+      <c r="P26" s="325"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="7">
@@ -13006,19 +13003,19 @@
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
-      <c r="I27" s="302" t="s">
+      <c r="I27" s="400" t="s">
         <v>665</v>
       </c>
-      <c r="J27" s="302" t="s">
+      <c r="J27" s="400" t="s">
         <v>668</v>
       </c>
-      <c r="K27" s="303" t="s">
+      <c r="K27" s="401" t="s">
         <v>671</v>
       </c>
       <c r="M27" s="11"/>
       <c r="N27" s="9"/>
       <c r="O27" s="242"/>
-      <c r="P27" s="342"/>
+      <c r="P27" s="325"/>
     </row>
     <row r="28" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
@@ -13036,22 +13033,22 @@
         <f t="shared" si="2"/>
         <v>6.25E-2</v>
       </c>
-      <c r="E28" s="344" t="s">
+      <c r="E28" s="318" t="s">
         <v>56</v>
       </c>
-      <c r="F28" s="345"/>
-      <c r="G28" s="345"/>
-      <c r="H28" s="345"/>
-      <c r="I28" s="345"/>
-      <c r="J28" s="345"/>
-      <c r="K28" s="345"/>
-      <c r="L28" s="345"/>
-      <c r="M28" s="346"/>
-      <c r="N28" s="350" t="s">
+      <c r="F28" s="319"/>
+      <c r="G28" s="319"/>
+      <c r="H28" s="319"/>
+      <c r="I28" s="319"/>
+      <c r="J28" s="319"/>
+      <c r="K28" s="319"/>
+      <c r="L28" s="319"/>
+      <c r="M28" s="320"/>
+      <c r="N28" s="330" t="s">
         <v>283</v>
       </c>
-      <c r="O28" s="351"/>
-      <c r="P28" s="342"/>
+      <c r="O28" s="331"/>
+      <c r="P28" s="325"/>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="7">
@@ -13090,13 +13087,13 @@
       <c r="K29" s="8"/>
       <c r="L29" s="8"/>
       <c r="M29" s="8"/>
-      <c r="N29" s="357" t="s">
+      <c r="N29" s="335" t="s">
         <v>312</v>
       </c>
-      <c r="O29" s="354" t="s">
+      <c r="O29" s="332" t="s">
         <v>353</v>
       </c>
-      <c r="P29" s="342"/>
+      <c r="P29" s="325"/>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
@@ -13133,15 +13130,15 @@
         <v>296</v>
       </c>
       <c r="K30" s="11"/>
-      <c r="L30" s="352" t="s">
+      <c r="L30" s="316" t="s">
         <v>228</v>
       </c>
-      <c r="M30" s="352" t="s">
+      <c r="M30" s="316" t="s">
         <v>229</v>
       </c>
-      <c r="N30" s="319"/>
-      <c r="O30" s="355"/>
-      <c r="P30" s="342"/>
+      <c r="N30" s="312"/>
+      <c r="O30" s="333"/>
+      <c r="P30" s="325"/>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="7">
@@ -13178,33 +13175,33 @@
         <v>303</v>
       </c>
       <c r="K31" s="104"/>
-      <c r="L31" s="353"/>
-      <c r="M31" s="353"/>
+      <c r="L31" s="317"/>
+      <c r="M31" s="317"/>
       <c r="N31" s="105" t="s">
         <v>311</v>
       </c>
-      <c r="O31" s="355"/>
-      <c r="P31" s="342"/>
+      <c r="O31" s="333"/>
+      <c r="P31" s="325"/>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
       <c r="B32" s="8"/>
       <c r="C32" s="103"/>
       <c r="D32" s="103"/>
-      <c r="E32" s="344" t="s">
+      <c r="E32" s="318" t="s">
         <v>681</v>
       </c>
-      <c r="F32" s="345"/>
-      <c r="G32" s="345"/>
-      <c r="H32" s="345"/>
-      <c r="I32" s="345"/>
-      <c r="J32" s="345"/>
-      <c r="K32" s="345"/>
-      <c r="L32" s="345"/>
-      <c r="M32" s="346"/>
+      <c r="F32" s="319"/>
+      <c r="G32" s="319"/>
+      <c r="H32" s="319"/>
+      <c r="I32" s="319"/>
+      <c r="J32" s="319"/>
+      <c r="K32" s="319"/>
+      <c r="L32" s="319"/>
+      <c r="M32" s="320"/>
       <c r="N32" s="105"/>
-      <c r="O32" s="355"/>
-      <c r="P32" s="342"/>
+      <c r="O32" s="333"/>
+      <c r="P32" s="325"/>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="7">
@@ -13237,11 +13234,11 @@
       <c r="K33" s="104"/>
       <c r="L33" s="8"/>
       <c r="M33" s="8"/>
-      <c r="N33" s="357" t="s">
+      <c r="N33" s="335" t="s">
         <v>354</v>
       </c>
-      <c r="O33" s="355"/>
-      <c r="P33" s="342"/>
+      <c r="O33" s="333"/>
+      <c r="P33" s="325"/>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="7">
@@ -13272,15 +13269,15 @@
       </c>
       <c r="J34" s="251"/>
       <c r="K34" s="104"/>
-      <c r="L34" s="352" t="s">
+      <c r="L34" s="316" t="s">
         <v>314</v>
       </c>
-      <c r="M34" s="352" t="s">
+      <c r="M34" s="316" t="s">
         <v>232</v>
       </c>
-      <c r="N34" s="365"/>
-      <c r="O34" s="355"/>
-      <c r="P34" s="342"/>
+      <c r="N34" s="340"/>
+      <c r="O34" s="333"/>
+      <c r="P34" s="325"/>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
@@ -13298,20 +13295,20 @@
         <f t="shared" si="2"/>
         <v>2.083333333333337E-2</v>
       </c>
-      <c r="E35" s="358" t="s">
+      <c r="E35" s="336" t="s">
         <v>310</v>
       </c>
-      <c r="F35" s="359"/>
-      <c r="G35" s="359"/>
-      <c r="H35" s="359"/>
-      <c r="I35" s="359"/>
-      <c r="J35" s="359"/>
-      <c r="K35" s="360"/>
-      <c r="L35" s="353"/>
-      <c r="M35" s="353"/>
+      <c r="F35" s="337"/>
+      <c r="G35" s="337"/>
+      <c r="H35" s="337"/>
+      <c r="I35" s="337"/>
+      <c r="J35" s="337"/>
+      <c r="K35" s="338"/>
+      <c r="L35" s="317"/>
+      <c r="M35" s="317"/>
       <c r="N35" s="105"/>
-      <c r="O35" s="356"/>
-      <c r="P35" s="343"/>
+      <c r="O35" s="334"/>
+      <c r="P35" s="326"/>
     </row>
     <row r="36" spans="1:16" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="12">
@@ -13328,17 +13325,17 @@
       <c r="D36" s="13">
         <v>2.083333333333337E-2</v>
       </c>
-      <c r="E36" s="366" t="s">
+      <c r="E36" s="321" t="s">
         <v>272</v>
       </c>
-      <c r="F36" s="367"/>
-      <c r="G36" s="367"/>
-      <c r="H36" s="367"/>
-      <c r="I36" s="367"/>
-      <c r="J36" s="367"/>
-      <c r="K36" s="367"/>
-      <c r="L36" s="367"/>
-      <c r="M36" s="368"/>
+      <c r="F36" s="322"/>
+      <c r="G36" s="322"/>
+      <c r="H36" s="322"/>
+      <c r="I36" s="322"/>
+      <c r="J36" s="322"/>
+      <c r="K36" s="322"/>
+      <c r="L36" s="322"/>
+      <c r="M36" s="323"/>
       <c r="N36" s="108" t="s">
         <v>396</v>
       </c>
@@ -13364,11 +13361,18 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="L30:L31"/>
-    <mergeCell ref="M30:M31"/>
-    <mergeCell ref="E32:M32"/>
-    <mergeCell ref="E36:M36"/>
-    <mergeCell ref="E11:M11"/>
+    <mergeCell ref="E8:K8"/>
+    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A4:P4"/>
+    <mergeCell ref="A5:P5"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="D7:D9"/>
+    <mergeCell ref="E7:M7"/>
+    <mergeCell ref="N7:N9"/>
+    <mergeCell ref="O7:P9"/>
+    <mergeCell ref="L8:M8"/>
     <mergeCell ref="P11:P35"/>
     <mergeCell ref="E28:M28"/>
     <mergeCell ref="O12:O24"/>
@@ -13385,18 +13389,11 @@
     <mergeCell ref="M34:M35"/>
     <mergeCell ref="E16:M16"/>
     <mergeCell ref="E21:M21"/>
-    <mergeCell ref="E8:K8"/>
-    <mergeCell ref="A3:P3"/>
-    <mergeCell ref="A4:P4"/>
-    <mergeCell ref="A5:P5"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="D7:D9"/>
-    <mergeCell ref="E7:M7"/>
-    <mergeCell ref="N7:N9"/>
-    <mergeCell ref="O7:P9"/>
-    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L30:L31"/>
+    <mergeCell ref="M30:M31"/>
+    <mergeCell ref="E32:M32"/>
+    <mergeCell ref="E36:M36"/>
+    <mergeCell ref="E11:M11"/>
   </mergeCells>
   <phoneticPr fontId="25" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -13417,58 +13414,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="371" t="s">
+      <c r="A1" s="361" t="s">
         <v>647</v>
       </c>
-      <c r="B1" s="371"/>
-      <c r="C1" s="371"/>
-      <c r="D1" s="371"/>
-      <c r="E1" s="371"/>
-      <c r="F1" s="371"/>
-      <c r="G1" s="371"/>
-      <c r="H1" s="371"/>
-      <c r="I1" s="371"/>
-      <c r="J1" s="371"/>
-      <c r="K1" s="371"/>
-      <c r="L1" s="371"/>
-      <c r="M1" s="371"/>
-      <c r="N1" s="371"/>
-      <c r="O1" s="371"/>
-      <c r="P1" s="371"/>
+      <c r="B1" s="361"/>
+      <c r="C1" s="361"/>
+      <c r="D1" s="361"/>
+      <c r="E1" s="361"/>
+      <c r="F1" s="361"/>
+      <c r="G1" s="361"/>
+      <c r="H1" s="361"/>
+      <c r="I1" s="361"/>
+      <c r="J1" s="361"/>
+      <c r="K1" s="361"/>
+      <c r="L1" s="361"/>
+      <c r="M1" s="361"/>
+      <c r="N1" s="361"/>
+      <c r="O1" s="361"/>
+      <c r="P1" s="361"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="369" t="s">
+      <c r="A2" s="359" t="s">
         <v>614</v>
       </c>
-      <c r="B2" s="370"/>
-      <c r="C2" s="369" t="s">
+      <c r="B2" s="360"/>
+      <c r="C2" s="359" t="s">
         <v>619</v>
       </c>
-      <c r="D2" s="370"/>
-      <c r="E2" s="369" t="s">
+      <c r="D2" s="360"/>
+      <c r="E2" s="359" t="s">
         <v>629</v>
       </c>
-      <c r="F2" s="370"/>
-      <c r="G2" s="369" t="s">
+      <c r="F2" s="360"/>
+      <c r="G2" s="359" t="s">
         <v>630</v>
       </c>
-      <c r="H2" s="370"/>
-      <c r="I2" s="369" t="s">
+      <c r="H2" s="360"/>
+      <c r="I2" s="359" t="s">
         <v>634</v>
       </c>
-      <c r="J2" s="370"/>
-      <c r="K2" s="369" t="s">
+      <c r="J2" s="360"/>
+      <c r="K2" s="359" t="s">
         <v>644</v>
       </c>
-      <c r="L2" s="370"/>
-      <c r="M2" s="369" t="s">
+      <c r="L2" s="360"/>
+      <c r="M2" s="359" t="s">
         <v>645</v>
       </c>
-      <c r="N2" s="370"/>
-      <c r="O2" s="369" t="s">
+      <c r="N2" s="360"/>
+      <c r="O2" s="359" t="s">
         <v>646</v>
       </c>
-      <c r="P2" s="370"/>
+      <c r="P2" s="360"/>
     </row>
     <row r="3" spans="1:16" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="247" t="s">
@@ -13727,60 +13724,55 @@
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="308" t="s">
+      <c r="A12" s="310" t="s">
         <v>279</v>
       </c>
-      <c r="B12" s="308"/>
-      <c r="C12" s="308" t="s">
+      <c r="B12" s="310"/>
+      <c r="C12" s="310" t="s">
         <v>280</v>
       </c>
-      <c r="D12" s="308"/>
-      <c r="E12" s="308" t="s">
+      <c r="D12" s="310"/>
+      <c r="E12" s="310" t="s">
         <v>281</v>
       </c>
-      <c r="F12" s="308"/>
-      <c r="G12" s="308" t="s">
+      <c r="F12" s="310"/>
+      <c r="G12" s="310" t="s">
         <v>282</v>
       </c>
-      <c r="H12" s="308"/>
+      <c r="H12" s="310"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="308" t="s">
+      <c r="A13" s="310" t="s">
         <v>228</v>
       </c>
-      <c r="B13" s="308"/>
-      <c r="C13" s="308"/>
-      <c r="D13" s="308"/>
-      <c r="E13" s="308" t="s">
+      <c r="B13" s="310"/>
+      <c r="C13" s="310"/>
+      <c r="D13" s="310"/>
+      <c r="E13" s="310" t="s">
         <v>229</v>
       </c>
-      <c r="F13" s="308"/>
-      <c r="G13" s="308"/>
-      <c r="H13" s="308"/>
+      <c r="F13" s="310"/>
+      <c r="G13" s="310"/>
+      <c r="H13" s="310"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C14" s="308" t="s">
+      <c r="C14" s="310" t="s">
         <v>233</v>
       </c>
-      <c r="D14" s="308"/>
-      <c r="E14" s="308"/>
-      <c r="F14" s="308"/>
+      <c r="D14" s="310"/>
+      <c r="E14" s="310"/>
+      <c r="F14" s="310"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C15" s="308" t="s">
+      <c r="C15" s="310" t="s">
         <v>232</v>
       </c>
-      <c r="D15" s="308"/>
-      <c r="E15" s="308"/>
-      <c r="F15" s="308"/>
+      <c r="D15" s="310"/>
+      <c r="E15" s="310"/>
+      <c r="F15" s="310"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="E13:H13"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="M2:N2"/>
     <mergeCell ref="O2:P2"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A12:B12"/>
@@ -13793,6 +13785,11 @@
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="K2:L2"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="E13:H13"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="M2:N2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13819,40 +13816,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="372" t="s">
+      <c r="A1" s="377" t="s">
         <v>586</v>
       </c>
-      <c r="B1" s="372"/>
-      <c r="C1" s="372"/>
-      <c r="D1" s="372"/>
-      <c r="E1" s="372"/>
-      <c r="F1" s="372"/>
-      <c r="G1" s="372"/>
-      <c r="H1" s="372"/>
-      <c r="I1" s="372"/>
-      <c r="J1" s="372"/>
+      <c r="B1" s="377"/>
+      <c r="C1" s="377"/>
+      <c r="D1" s="377"/>
+      <c r="E1" s="377"/>
+      <c r="F1" s="377"/>
+      <c r="G1" s="377"/>
+      <c r="H1" s="377"/>
+      <c r="I1" s="377"/>
+      <c r="J1" s="377"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="373" t="s">
+      <c r="A2" s="378" t="s">
         <v>605</v>
       </c>
-      <c r="B2" s="374"/>
-      <c r="C2" s="375" t="s">
+      <c r="B2" s="379"/>
+      <c r="C2" s="380" t="s">
         <v>606</v>
       </c>
-      <c r="D2" s="376"/>
-      <c r="E2" s="373" t="s">
+      <c r="D2" s="381"/>
+      <c r="E2" s="378" t="s">
         <v>607</v>
       </c>
-      <c r="F2" s="374"/>
-      <c r="G2" s="375" t="s">
+      <c r="F2" s="379"/>
+      <c r="G2" s="380" t="s">
         <v>571</v>
       </c>
-      <c r="H2" s="376"/>
-      <c r="I2" s="373" t="s">
+      <c r="H2" s="381"/>
+      <c r="I2" s="378" t="s">
         <v>572</v>
       </c>
-      <c r="J2" s="374"/>
+      <c r="J2" s="379"/>
     </row>
     <row r="3" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="222" t="s">
@@ -13890,13 +13887,13 @@
       <c r="A4" s="224" t="s">
         <v>587</v>
       </c>
-      <c r="B4" s="377" t="s">
+      <c r="B4" s="373" t="s">
         <v>399</v>
       </c>
       <c r="C4" s="188" t="s">
         <v>415</v>
       </c>
-      <c r="D4" s="379" t="s">
+      <c r="D4" s="374" t="s">
         <v>449</v>
       </c>
       <c r="E4" s="224" t="s">
@@ -13908,13 +13905,13 @@
       <c r="G4" s="188" t="s">
         <v>465</v>
       </c>
-      <c r="H4" s="381" t="s">
+      <c r="H4" s="375" t="s">
         <v>567</v>
       </c>
       <c r="I4" s="197" t="s">
         <v>573</v>
       </c>
-      <c r="J4" s="383" t="s">
+      <c r="J4" s="371" t="s">
         <v>577</v>
       </c>
     </row>
@@ -13922,11 +13919,11 @@
       <c r="A5" s="225" t="s">
         <v>588</v>
       </c>
-      <c r="B5" s="378"/>
+      <c r="B5" s="362"/>
       <c r="C5" s="185" t="s">
         <v>416</v>
       </c>
-      <c r="D5" s="380"/>
+      <c r="D5" s="364"/>
       <c r="E5" s="225" t="s">
         <v>498</v>
       </c>
@@ -13936,23 +13933,23 @@
       <c r="G5" s="186" t="s">
         <v>534</v>
       </c>
-      <c r="H5" s="382"/>
+      <c r="H5" s="366"/>
       <c r="I5" s="195" t="s">
         <v>574</v>
       </c>
-      <c r="J5" s="384"/>
+      <c r="J5" s="376"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="225" t="s">
         <v>589</v>
       </c>
-      <c r="B6" s="378" t="s">
+      <c r="B6" s="362" t="s">
         <v>400</v>
       </c>
       <c r="C6" s="185" t="s">
         <v>417</v>
       </c>
-      <c r="D6" s="380" t="s">
+      <c r="D6" s="364" t="s">
         <v>450</v>
       </c>
       <c r="E6" s="225" t="s">
@@ -13964,13 +13961,13 @@
       <c r="G6" s="185" t="s">
         <v>498</v>
       </c>
-      <c r="H6" s="382" t="s">
+      <c r="H6" s="366" t="s">
         <v>568</v>
       </c>
       <c r="I6" s="195" t="s">
         <v>575</v>
       </c>
-      <c r="J6" s="384" t="s">
+      <c r="J6" s="376" t="s">
         <v>578</v>
       </c>
     </row>
@@ -13978,11 +13975,11 @@
       <c r="A7" s="225" t="s">
         <v>590</v>
       </c>
-      <c r="B7" s="378"/>
+      <c r="B7" s="362"/>
       <c r="C7" s="185" t="s">
         <v>418</v>
       </c>
-      <c r="D7" s="380"/>
+      <c r="D7" s="364"/>
       <c r="E7" s="225" t="s">
         <v>500</v>
       </c>
@@ -13992,35 +13989,35 @@
       <c r="G7" s="186" t="s">
         <v>533</v>
       </c>
-      <c r="H7" s="382"/>
+      <c r="H7" s="366"/>
       <c r="I7" s="195" t="s">
         <v>576</v>
       </c>
-      <c r="J7" s="384"/>
+      <c r="J7" s="376"/>
     </row>
     <row r="8" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="225" t="s">
         <v>591</v>
       </c>
-      <c r="B8" s="378" t="s">
+      <c r="B8" s="362" t="s">
         <v>401</v>
       </c>
       <c r="C8" s="185" t="s">
         <v>419</v>
       </c>
-      <c r="D8" s="380" t="s">
+      <c r="D8" s="364" t="s">
         <v>451</v>
       </c>
       <c r="E8" s="225" t="s">
         <v>559</v>
       </c>
-      <c r="F8" s="385" t="s">
+      <c r="F8" s="368" t="s">
         <v>523</v>
       </c>
       <c r="G8" s="185" t="s">
         <v>499</v>
       </c>
-      <c r="H8" s="382" t="s">
+      <c r="H8" s="366" t="s">
         <v>569</v>
       </c>
       <c r="I8" s="236"/>
@@ -14030,53 +14027,53 @@
       <c r="A9" s="225" t="s">
         <v>592</v>
       </c>
-      <c r="B9" s="378"/>
+      <c r="B9" s="362"/>
       <c r="C9" s="185" t="s">
         <v>420</v>
       </c>
-      <c r="D9" s="380"/>
+      <c r="D9" s="364"/>
       <c r="E9" s="225" t="s">
         <v>560</v>
       </c>
-      <c r="F9" s="385"/>
+      <c r="F9" s="368"/>
       <c r="G9" s="186" t="s">
         <v>532</v>
       </c>
-      <c r="H9" s="382"/>
-      <c r="I9" s="386" t="s">
+      <c r="H9" s="366"/>
+      <c r="I9" s="369" t="s">
         <v>579</v>
       </c>
-      <c r="J9" s="387"/>
+      <c r="J9" s="370"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="225" t="s">
         <v>593</v>
       </c>
-      <c r="B10" s="378" t="s">
+      <c r="B10" s="362" t="s">
         <v>402</v>
       </c>
       <c r="C10" s="185" t="s">
         <v>421</v>
       </c>
-      <c r="D10" s="380" t="s">
+      <c r="D10" s="364" t="s">
         <v>452</v>
       </c>
       <c r="E10" s="225" t="s">
         <v>561</v>
       </c>
-      <c r="F10" s="385" t="s">
+      <c r="F10" s="368" t="s">
         <v>524</v>
       </c>
       <c r="G10" s="185" t="s">
         <v>500</v>
       </c>
-      <c r="H10" s="382" t="s">
+      <c r="H10" s="366" t="s">
         <v>570</v>
       </c>
       <c r="I10" s="197" t="s">
         <v>580</v>
       </c>
-      <c r="J10" s="383" t="s">
+      <c r="J10" s="371" t="s">
         <v>233</v>
       </c>
     </row>
@@ -14084,45 +14081,45 @@
       <c r="A11" s="225" t="s">
         <v>594</v>
       </c>
-      <c r="B11" s="378"/>
+      <c r="B11" s="362"/>
       <c r="C11" s="185" t="s">
         <v>422</v>
       </c>
-      <c r="D11" s="380"/>
+      <c r="D11" s="364"/>
       <c r="E11" s="225" t="s">
         <v>562</v>
       </c>
-      <c r="F11" s="385"/>
+      <c r="F11" s="368"/>
       <c r="G11" s="186" t="s">
         <v>531</v>
       </c>
-      <c r="H11" s="382"/>
+      <c r="H11" s="366"/>
       <c r="I11" s="196" t="s">
         <v>581</v>
       </c>
-      <c r="J11" s="388"/>
+      <c r="J11" s="372"/>
     </row>
     <row r="12" spans="1:10" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="225" t="s">
         <v>595</v>
       </c>
-      <c r="B12" s="378" t="s">
+      <c r="B12" s="362" t="s">
         <v>403</v>
       </c>
       <c r="C12" s="185" t="s">
         <v>431</v>
       </c>
-      <c r="D12" s="380" t="s">
+      <c r="D12" s="364" t="s">
         <v>453</v>
       </c>
       <c r="E12" s="225" t="s">
         <v>501</v>
       </c>
-      <c r="F12" s="385" t="s">
+      <c r="F12" s="368" t="s">
         <v>525</v>
       </c>
       <c r="G12" s="185"/>
-      <c r="H12" s="382"/>
+      <c r="H12" s="366"/>
       <c r="I12" s="238"/>
       <c r="J12" s="239"/>
     </row>
@@ -14130,47 +14127,47 @@
       <c r="A13" s="225" t="s">
         <v>596</v>
       </c>
-      <c r="B13" s="378"/>
+      <c r="B13" s="362"/>
       <c r="C13" s="185" t="s">
         <v>432</v>
       </c>
-      <c r="D13" s="380"/>
+      <c r="D13" s="364"/>
       <c r="E13" s="225" t="s">
         <v>502</v>
       </c>
-      <c r="F13" s="385"/>
+      <c r="F13" s="368"/>
       <c r="G13" s="195"/>
-      <c r="H13" s="382"/>
-      <c r="I13" s="386" t="s">
+      <c r="H13" s="366"/>
+      <c r="I13" s="369" t="s">
         <v>582</v>
       </c>
-      <c r="J13" s="387"/>
+      <c r="J13" s="370"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="225" t="s">
         <v>597</v>
       </c>
-      <c r="B14" s="378" t="s">
+      <c r="B14" s="362" t="s">
         <v>404</v>
       </c>
       <c r="C14" s="185" t="s">
         <v>433</v>
       </c>
-      <c r="D14" s="380" t="s">
+      <c r="D14" s="364" t="s">
         <v>454</v>
       </c>
       <c r="E14" s="225" t="s">
         <v>503</v>
       </c>
-      <c r="F14" s="385" t="s">
+      <c r="F14" s="368" t="s">
         <v>526</v>
       </c>
       <c r="G14" s="185"/>
-      <c r="H14" s="382"/>
+      <c r="H14" s="366"/>
       <c r="I14" s="197" t="s">
         <v>583</v>
       </c>
-      <c r="J14" s="383" t="s">
+      <c r="J14" s="371" t="s">
         <v>232</v>
       </c>
     </row>
@@ -14178,33 +14175,33 @@
       <c r="A15" s="225" t="s">
         <v>598</v>
       </c>
-      <c r="B15" s="378"/>
+      <c r="B15" s="362"/>
       <c r="C15" s="185" t="s">
         <v>434</v>
       </c>
-      <c r="D15" s="380"/>
+      <c r="D15" s="364"/>
       <c r="E15" s="225" t="s">
         <v>504</v>
       </c>
-      <c r="F15" s="385"/>
+      <c r="F15" s="368"/>
       <c r="G15" s="195"/>
-      <c r="H15" s="382"/>
+      <c r="H15" s="366"/>
       <c r="I15" s="196" t="s">
         <v>584</v>
       </c>
-      <c r="J15" s="388"/>
+      <c r="J15" s="372"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="225" t="s">
         <v>599</v>
       </c>
-      <c r="B16" s="378" t="s">
+      <c r="B16" s="362" t="s">
         <v>405</v>
       </c>
       <c r="C16" s="185" t="s">
         <v>435</v>
       </c>
-      <c r="D16" s="380" t="s">
+      <c r="D16" s="364" t="s">
         <v>455</v>
       </c>
       <c r="E16" s="226" t="s">
@@ -14214,7 +14211,7 @@
         <v>514</v>
       </c>
       <c r="G16" s="185"/>
-      <c r="H16" s="382"/>
+      <c r="H16" s="366"/>
       <c r="I16" s="197"/>
       <c r="J16" s="240"/>
     </row>
@@ -14222,11 +14219,11 @@
       <c r="A17" s="225" t="s">
         <v>600</v>
       </c>
-      <c r="B17" s="378"/>
+      <c r="B17" s="362"/>
       <c r="C17" s="185" t="s">
         <v>436</v>
       </c>
-      <c r="D17" s="380"/>
+      <c r="D17" s="364"/>
       <c r="E17" s="226" t="s">
         <v>564</v>
       </c>
@@ -14234,7 +14231,7 @@
         <v>514</v>
       </c>
       <c r="G17" s="195"/>
-      <c r="H17" s="382"/>
+      <c r="H17" s="366"/>
       <c r="I17" s="195"/>
       <c r="J17" s="234"/>
     </row>
@@ -14242,13 +14239,13 @@
       <c r="A18" s="225" t="s">
         <v>601</v>
       </c>
-      <c r="B18" s="378" t="s">
+      <c r="B18" s="362" t="s">
         <v>406</v>
       </c>
       <c r="C18" s="185" t="s">
         <v>437</v>
       </c>
-      <c r="D18" s="380" t="s">
+      <c r="D18" s="364" t="s">
         <v>456</v>
       </c>
       <c r="E18" s="226" t="s">
@@ -14258,7 +14255,7 @@
         <v>514</v>
       </c>
       <c r="G18" s="185"/>
-      <c r="H18" s="382"/>
+      <c r="H18" s="366"/>
       <c r="I18" s="195"/>
       <c r="J18" s="234"/>
     </row>
@@ -14266,11 +14263,11 @@
       <c r="A19" s="232" t="s">
         <v>602</v>
       </c>
-      <c r="B19" s="389"/>
+      <c r="B19" s="363"/>
       <c r="C19" s="233" t="s">
         <v>438</v>
       </c>
-      <c r="D19" s="390"/>
+      <c r="D19" s="365"/>
       <c r="E19" s="227" t="s">
         <v>566</v>
       </c>
@@ -14278,22 +14275,26 @@
         <v>514</v>
       </c>
       <c r="G19" s="196"/>
-      <c r="H19" s="391"/>
+      <c r="H19" s="367"/>
       <c r="I19" s="196"/>
       <c r="J19" s="235"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="J6:J7"/>
     <mergeCell ref="F8:F9"/>
     <mergeCell ref="H12:H13"/>
     <mergeCell ref="I13:J13"/>
@@ -14310,20 +14311,16 @@
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="H10:H11"/>
     <mergeCell ref="J10:J11"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="H16:H17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -14353,46 +14350,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="398" t="s">
+      <c r="A1" s="382" t="s">
         <v>398</v>
       </c>
-      <c r="B1" s="398"/>
-      <c r="C1" s="398"/>
-      <c r="D1" s="398"/>
-      <c r="E1" s="398"/>
-      <c r="F1" s="398"/>
-      <c r="G1" s="398"/>
-      <c r="H1" s="398"/>
-      <c r="I1" s="398"/>
-      <c r="J1" s="398"/>
-      <c r="K1" s="398"/>
-      <c r="L1" s="398"/>
+      <c r="B1" s="382"/>
+      <c r="C1" s="382"/>
+      <c r="D1" s="382"/>
+      <c r="E1" s="382"/>
+      <c r="F1" s="382"/>
+      <c r="G1" s="382"/>
+      <c r="H1" s="382"/>
+      <c r="I1" s="382"/>
+      <c r="J1" s="382"/>
+      <c r="K1" s="382"/>
+      <c r="L1" s="382"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="395" t="s">
+      <c r="A2" s="385" t="s">
         <v>539</v>
       </c>
-      <c r="B2" s="396"/>
-      <c r="C2" s="375" t="s">
+      <c r="B2" s="386"/>
+      <c r="C2" s="380" t="s">
         <v>540</v>
       </c>
-      <c r="D2" s="376"/>
-      <c r="E2" s="395" t="s">
+      <c r="D2" s="381"/>
+      <c r="E2" s="385" t="s">
         <v>541</v>
       </c>
-      <c r="F2" s="396"/>
-      <c r="G2" s="375" t="s">
+      <c r="F2" s="386"/>
+      <c r="G2" s="380" t="s">
         <v>550</v>
       </c>
-      <c r="H2" s="376"/>
-      <c r="I2" s="395" t="s">
+      <c r="H2" s="381"/>
+      <c r="I2" s="385" t="s">
         <v>571</v>
       </c>
-      <c r="J2" s="396"/>
-      <c r="K2" s="395" t="s">
+      <c r="J2" s="386"/>
+      <c r="K2" s="385" t="s">
         <v>572</v>
       </c>
-      <c r="L2" s="396"/>
+      <c r="L2" s="386"/>
     </row>
     <row r="3" spans="1:12" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="191" t="s">
@@ -14436,13 +14433,13 @@
       <c r="A4" s="183" t="s">
         <v>466</v>
       </c>
-      <c r="B4" s="397" t="s">
+      <c r="B4" s="391" t="s">
         <v>399</v>
       </c>
       <c r="C4" s="188" t="s">
         <v>415</v>
       </c>
-      <c r="D4" s="379" t="s">
+      <c r="D4" s="374" t="s">
         <v>449</v>
       </c>
       <c r="E4" s="183" t="s">
@@ -14454,19 +14451,19 @@
       <c r="G4" s="188" t="s">
         <v>465</v>
       </c>
-      <c r="H4" s="381" t="s">
+      <c r="H4" s="375" t="s">
         <v>542</v>
       </c>
       <c r="I4" s="190" t="s">
         <v>551</v>
       </c>
-      <c r="J4" s="401" t="s">
+      <c r="J4" s="387" t="s">
         <v>567</v>
       </c>
       <c r="K4" s="197" t="s">
         <v>573</v>
       </c>
-      <c r="L4" s="383" t="s">
+      <c r="L4" s="371" t="s">
         <v>577</v>
       </c>
     </row>
@@ -14474,11 +14471,11 @@
       <c r="A5" s="180" t="s">
         <v>467</v>
       </c>
-      <c r="B5" s="392"/>
+      <c r="B5" s="390"/>
       <c r="C5" s="185" t="s">
         <v>416</v>
       </c>
-      <c r="D5" s="380"/>
+      <c r="D5" s="364"/>
       <c r="E5" s="180" t="s">
         <v>498</v>
       </c>
@@ -14488,27 +14485,27 @@
       <c r="G5" s="186" t="s">
         <v>538</v>
       </c>
-      <c r="H5" s="382"/>
+      <c r="H5" s="366"/>
       <c r="I5" s="181" t="s">
         <v>552</v>
       </c>
-      <c r="J5" s="393"/>
+      <c r="J5" s="388"/>
       <c r="K5" s="195" t="s">
         <v>574</v>
       </c>
-      <c r="L5" s="384"/>
+      <c r="L5" s="376"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="180" t="s">
         <v>468</v>
       </c>
-      <c r="B6" s="392" t="s">
+      <c r="B6" s="390" t="s">
         <v>400</v>
       </c>
       <c r="C6" s="185" t="s">
         <v>417</v>
       </c>
-      <c r="D6" s="380" t="s">
+      <c r="D6" s="364" t="s">
         <v>450</v>
       </c>
       <c r="E6" s="180" t="s">
@@ -14520,19 +14517,19 @@
       <c r="G6" s="185" t="s">
         <v>498</v>
       </c>
-      <c r="H6" s="382" t="s">
+      <c r="H6" s="366" t="s">
         <v>543</v>
       </c>
       <c r="I6" s="181" t="s">
         <v>553</v>
       </c>
-      <c r="J6" s="393" t="s">
+      <c r="J6" s="388" t="s">
         <v>568</v>
       </c>
       <c r="K6" s="195" t="s">
         <v>575</v>
       </c>
-      <c r="L6" s="384" t="s">
+      <c r="L6" s="376" t="s">
         <v>578</v>
       </c>
     </row>
@@ -14540,11 +14537,11 @@
       <c r="A7" s="180" t="s">
         <v>469</v>
       </c>
-      <c r="B7" s="392"/>
+      <c r="B7" s="390"/>
       <c r="C7" s="185" t="s">
         <v>418</v>
       </c>
-      <c r="D7" s="380"/>
+      <c r="D7" s="364"/>
       <c r="E7" s="180" t="s">
         <v>500</v>
       </c>
@@ -14554,27 +14551,27 @@
       <c r="G7" s="186" t="s">
         <v>537</v>
       </c>
-      <c r="H7" s="382"/>
+      <c r="H7" s="366"/>
       <c r="I7" s="181" t="s">
         <v>554</v>
       </c>
-      <c r="J7" s="393"/>
+      <c r="J7" s="388"/>
       <c r="K7" s="196" t="s">
         <v>576</v>
       </c>
-      <c r="L7" s="388"/>
+      <c r="L7" s="372"/>
     </row>
     <row r="8" spans="1:12" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="180" t="s">
         <v>470</v>
       </c>
-      <c r="B8" s="392" t="s">
+      <c r="B8" s="390" t="s">
         <v>401</v>
       </c>
       <c r="C8" s="185" t="s">
         <v>419</v>
       </c>
-      <c r="D8" s="380" t="s">
+      <c r="D8" s="364" t="s">
         <v>451</v>
       </c>
       <c r="E8" s="180" t="s">
@@ -14586,13 +14583,13 @@
       <c r="G8" s="185" t="s">
         <v>499</v>
       </c>
-      <c r="H8" s="382" t="s">
+      <c r="H8" s="366" t="s">
         <v>544</v>
       </c>
       <c r="I8" s="181" t="s">
         <v>555</v>
       </c>
-      <c r="J8" s="393" t="s">
+      <c r="J8" s="388" t="s">
         <v>569</v>
       </c>
       <c r="K8" s="168"/>
@@ -14602,11 +14599,11 @@
       <c r="A9" s="180" t="s">
         <v>471</v>
       </c>
-      <c r="B9" s="392"/>
+      <c r="B9" s="390"/>
       <c r="C9" s="185" t="s">
         <v>420</v>
       </c>
-      <c r="D9" s="380"/>
+      <c r="D9" s="364"/>
       <c r="E9" s="180" t="s">
         <v>502</v>
       </c>
@@ -14616,27 +14613,27 @@
       <c r="G9" s="186" t="s">
         <v>536</v>
       </c>
-      <c r="H9" s="382"/>
+      <c r="H9" s="366"/>
       <c r="I9" s="181" t="s">
         <v>556</v>
       </c>
-      <c r="J9" s="393"/>
-      <c r="K9" s="399" t="s">
+      <c r="J9" s="388"/>
+      <c r="K9" s="383" t="s">
         <v>579</v>
       </c>
-      <c r="L9" s="400"/>
+      <c r="L9" s="384"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="180" t="s">
         <v>472</v>
       </c>
-      <c r="B10" s="392" t="s">
+      <c r="B10" s="390" t="s">
         <v>402</v>
       </c>
       <c r="C10" s="185" t="s">
         <v>421</v>
       </c>
-      <c r="D10" s="380" t="s">
+      <c r="D10" s="364" t="s">
         <v>452</v>
       </c>
       <c r="E10" s="180" t="s">
@@ -14648,19 +14645,19 @@
       <c r="G10" s="185" t="s">
         <v>500</v>
       </c>
-      <c r="H10" s="382" t="s">
+      <c r="H10" s="366" t="s">
         <v>545</v>
       </c>
       <c r="I10" s="181" t="s">
         <v>557</v>
       </c>
-      <c r="J10" s="393" t="s">
+      <c r="J10" s="388" t="s">
         <v>570</v>
       </c>
       <c r="K10" s="197" t="s">
         <v>580</v>
       </c>
-      <c r="L10" s="383" t="s">
+      <c r="L10" s="371" t="s">
         <v>233</v>
       </c>
     </row>
@@ -14668,11 +14665,11 @@
       <c r="A11" s="180" t="s">
         <v>473</v>
       </c>
-      <c r="B11" s="392"/>
+      <c r="B11" s="390"/>
       <c r="C11" s="185" t="s">
         <v>422</v>
       </c>
-      <c r="D11" s="380"/>
+      <c r="D11" s="364"/>
       <c r="E11" s="180" t="s">
         <v>504</v>
       </c>
@@ -14682,39 +14679,39 @@
       <c r="G11" s="186" t="s">
         <v>535</v>
       </c>
-      <c r="H11" s="382"/>
+      <c r="H11" s="366"/>
       <c r="I11" s="182" t="s">
         <v>558</v>
       </c>
-      <c r="J11" s="394"/>
+      <c r="J11" s="389"/>
       <c r="K11" s="196" t="s">
         <v>581</v>
       </c>
-      <c r="L11" s="388"/>
+      <c r="L11" s="372"/>
     </row>
     <row r="12" spans="1:12" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="180" t="s">
         <v>474</v>
       </c>
-      <c r="B12" s="392" t="s">
+      <c r="B12" s="390" t="s">
         <v>403</v>
       </c>
       <c r="C12" s="185" t="s">
         <v>423</v>
       </c>
-      <c r="D12" s="380" t="s">
+      <c r="D12" s="364" t="s">
         <v>453</v>
       </c>
       <c r="E12" s="180" t="s">
         <v>559</v>
       </c>
-      <c r="F12" s="393" t="s">
+      <c r="F12" s="388" t="s">
         <v>523</v>
       </c>
       <c r="G12" s="185" t="s">
         <v>501</v>
       </c>
-      <c r="H12" s="382" t="s">
+      <c r="H12" s="366" t="s">
         <v>546</v>
       </c>
       <c r="I12" s="175"/>
@@ -14726,49 +14723,49 @@
       <c r="A13" s="180" t="s">
         <v>475</v>
       </c>
-      <c r="B13" s="392"/>
+      <c r="B13" s="390"/>
       <c r="C13" s="185" t="s">
         <v>424</v>
       </c>
-      <c r="D13" s="380"/>
+      <c r="D13" s="364"/>
       <c r="E13" s="180" t="s">
         <v>560</v>
       </c>
-      <c r="F13" s="393"/>
+      <c r="F13" s="388"/>
       <c r="G13" s="186" t="s">
         <v>534</v>
       </c>
-      <c r="H13" s="382"/>
+      <c r="H13" s="366"/>
       <c r="I13" s="175"/>
       <c r="J13" s="177"/>
-      <c r="K13" s="399" t="s">
+      <c r="K13" s="383" t="s">
         <v>582</v>
       </c>
-      <c r="L13" s="400"/>
+      <c r="L13" s="384"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="180" t="s">
         <v>476</v>
       </c>
-      <c r="B14" s="392" t="s">
+      <c r="B14" s="390" t="s">
         <v>404</v>
       </c>
       <c r="C14" s="185" t="s">
         <v>425</v>
       </c>
-      <c r="D14" s="380" t="s">
+      <c r="D14" s="364" t="s">
         <v>454</v>
       </c>
       <c r="E14" s="180" t="s">
         <v>561</v>
       </c>
-      <c r="F14" s="393" t="s">
+      <c r="F14" s="388" t="s">
         <v>524</v>
       </c>
       <c r="G14" s="185" t="s">
         <v>502</v>
       </c>
-      <c r="H14" s="382" t="s">
+      <c r="H14" s="366" t="s">
         <v>547</v>
       </c>
       <c r="I14" s="175"/>
@@ -14776,7 +14773,7 @@
       <c r="K14" s="197" t="s">
         <v>583</v>
       </c>
-      <c r="L14" s="383" t="s">
+      <c r="L14" s="371" t="s">
         <v>232</v>
       </c>
     </row>
@@ -14784,49 +14781,49 @@
       <c r="A15" s="180" t="s">
         <v>477</v>
       </c>
-      <c r="B15" s="392"/>
+      <c r="B15" s="390"/>
       <c r="C15" s="185" t="s">
         <v>426</v>
       </c>
-      <c r="D15" s="380"/>
+      <c r="D15" s="364"/>
       <c r="E15" s="180" t="s">
         <v>562</v>
       </c>
-      <c r="F15" s="393"/>
+      <c r="F15" s="388"/>
       <c r="G15" s="186" t="s">
         <v>533</v>
       </c>
-      <c r="H15" s="382"/>
+      <c r="H15" s="366"/>
       <c r="I15" s="175"/>
       <c r="J15" s="177"/>
       <c r="K15" s="196" t="s">
         <v>584</v>
       </c>
-      <c r="L15" s="388"/>
+      <c r="L15" s="372"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="180" t="s">
         <v>478</v>
       </c>
-      <c r="B16" s="392" t="s">
+      <c r="B16" s="390" t="s">
         <v>405</v>
       </c>
       <c r="C16" s="185" t="s">
         <v>427</v>
       </c>
-      <c r="D16" s="380" t="s">
+      <c r="D16" s="364" t="s">
         <v>455</v>
       </c>
       <c r="E16" s="180" t="s">
         <v>563</v>
       </c>
-      <c r="F16" s="393" t="s">
+      <c r="F16" s="388" t="s">
         <v>525</v>
       </c>
       <c r="G16" s="185" t="s">
         <v>503</v>
       </c>
-      <c r="H16" s="382" t="s">
+      <c r="H16" s="366" t="s">
         <v>548</v>
       </c>
       <c r="I16" s="175"/>
@@ -14838,19 +14835,19 @@
       <c r="A17" s="180" t="s">
         <v>479</v>
       </c>
-      <c r="B17" s="392"/>
+      <c r="B17" s="390"/>
       <c r="C17" s="185" t="s">
         <v>428</v>
       </c>
-      <c r="D17" s="380"/>
+      <c r="D17" s="364"/>
       <c r="E17" s="180" t="s">
         <v>564</v>
       </c>
-      <c r="F17" s="393"/>
+      <c r="F17" s="388"/>
       <c r="G17" s="186" t="s">
         <v>532</v>
       </c>
-      <c r="H17" s="382"/>
+      <c r="H17" s="366"/>
       <c r="I17" s="175"/>
       <c r="J17" s="177"/>
       <c r="K17" s="168"/>
@@ -14860,25 +14857,25 @@
       <c r="A18" s="180" t="s">
         <v>480</v>
       </c>
-      <c r="B18" s="392" t="s">
+      <c r="B18" s="390" t="s">
         <v>406</v>
       </c>
       <c r="C18" s="185" t="s">
         <v>429</v>
       </c>
-      <c r="D18" s="380" t="s">
+      <c r="D18" s="364" t="s">
         <v>456</v>
       </c>
       <c r="E18" s="180" t="s">
         <v>565</v>
       </c>
-      <c r="F18" s="393" t="s">
+      <c r="F18" s="388" t="s">
         <v>526</v>
       </c>
       <c r="G18" s="185" t="s">
         <v>504</v>
       </c>
-      <c r="H18" s="382" t="s">
+      <c r="H18" s="366" t="s">
         <v>549</v>
       </c>
       <c r="I18" s="175"/>
@@ -14890,19 +14887,19 @@
       <c r="A19" s="180" t="s">
         <v>481</v>
       </c>
-      <c r="B19" s="392"/>
+      <c r="B19" s="390"/>
       <c r="C19" s="185" t="s">
         <v>430</v>
       </c>
-      <c r="D19" s="380"/>
+      <c r="D19" s="364"/>
       <c r="E19" s="180" t="s">
         <v>566</v>
       </c>
-      <c r="F19" s="393"/>
+      <c r="F19" s="388"/>
       <c r="G19" s="187" t="s">
         <v>531</v>
       </c>
-      <c r="H19" s="391"/>
+      <c r="H19" s="367"/>
       <c r="I19" s="175"/>
       <c r="J19" s="177"/>
       <c r="K19" s="168"/>
@@ -14912,19 +14909,19 @@
       <c r="A20" s="180" t="s">
         <v>482</v>
       </c>
-      <c r="B20" s="392" t="s">
+      <c r="B20" s="390" t="s">
         <v>407</v>
       </c>
       <c r="C20" s="185" t="s">
         <v>431</v>
       </c>
-      <c r="D20" s="380" t="s">
+      <c r="D20" s="364" t="s">
         <v>457</v>
       </c>
       <c r="E20" s="180" t="s">
         <v>515</v>
       </c>
-      <c r="F20" s="393" t="s">
+      <c r="F20" s="388" t="s">
         <v>527</v>
       </c>
       <c r="G20" s="170"/>
@@ -14938,15 +14935,15 @@
       <c r="A21" s="180" t="s">
         <v>483</v>
       </c>
-      <c r="B21" s="392"/>
+      <c r="B21" s="390"/>
       <c r="C21" s="185" t="s">
         <v>432</v>
       </c>
-      <c r="D21" s="380"/>
+      <c r="D21" s="364"/>
       <c r="E21" s="180" t="s">
         <v>516</v>
       </c>
-      <c r="F21" s="393"/>
+      <c r="F21" s="388"/>
       <c r="G21" s="170"/>
       <c r="H21" s="169"/>
       <c r="I21" s="175"/>
@@ -14958,19 +14955,19 @@
       <c r="A22" s="181" t="s">
         <v>484</v>
       </c>
-      <c r="B22" s="393" t="s">
+      <c r="B22" s="388" t="s">
         <v>408</v>
       </c>
       <c r="C22" s="186" t="s">
         <v>433</v>
       </c>
-      <c r="D22" s="382" t="s">
+      <c r="D22" s="366" t="s">
         <v>458</v>
       </c>
       <c r="E22" s="181" t="s">
         <v>517</v>
       </c>
-      <c r="F22" s="393" t="s">
+      <c r="F22" s="388" t="s">
         <v>528</v>
       </c>
       <c r="G22" s="170"/>
@@ -14984,15 +14981,15 @@
       <c r="A23" s="181" t="s">
         <v>485</v>
       </c>
-      <c r="B23" s="393"/>
+      <c r="B23" s="388"/>
       <c r="C23" s="186" t="s">
         <v>434</v>
       </c>
-      <c r="D23" s="382"/>
+      <c r="D23" s="366"/>
       <c r="E23" s="181" t="s">
         <v>518</v>
       </c>
-      <c r="F23" s="393"/>
+      <c r="F23" s="388"/>
       <c r="G23" s="170"/>
       <c r="H23" s="169"/>
       <c r="I23" s="175"/>
@@ -15004,19 +15001,19 @@
       <c r="A24" s="181" t="s">
         <v>486</v>
       </c>
-      <c r="B24" s="393" t="s">
+      <c r="B24" s="388" t="s">
         <v>409</v>
       </c>
       <c r="C24" s="186" t="s">
         <v>435</v>
       </c>
-      <c r="D24" s="382" t="s">
+      <c r="D24" s="366" t="s">
         <v>459</v>
       </c>
       <c r="E24" s="181" t="s">
         <v>519</v>
       </c>
-      <c r="F24" s="393" t="s">
+      <c r="F24" s="388" t="s">
         <v>529</v>
       </c>
       <c r="G24" s="170"/>
@@ -15030,15 +15027,15 @@
       <c r="A25" s="181" t="s">
         <v>487</v>
       </c>
-      <c r="B25" s="393"/>
+      <c r="B25" s="388"/>
       <c r="C25" s="186" t="s">
         <v>436</v>
       </c>
-      <c r="D25" s="382"/>
+      <c r="D25" s="366"/>
       <c r="E25" s="181" t="s">
         <v>520</v>
       </c>
-      <c r="F25" s="393"/>
+      <c r="F25" s="388"/>
       <c r="G25" s="170"/>
       <c r="H25" s="169"/>
       <c r="I25" s="175"/>
@@ -15050,19 +15047,19 @@
       <c r="A26" s="181" t="s">
         <v>488</v>
       </c>
-      <c r="B26" s="393" t="s">
+      <c r="B26" s="388" t="s">
         <v>410</v>
       </c>
       <c r="C26" s="186" t="s">
         <v>437</v>
       </c>
-      <c r="D26" s="382" t="s">
+      <c r="D26" s="366" t="s">
         <v>460</v>
       </c>
       <c r="E26" s="181" t="s">
         <v>521</v>
       </c>
-      <c r="F26" s="393" t="s">
+      <c r="F26" s="388" t="s">
         <v>530</v>
       </c>
       <c r="G26" s="171"/>
@@ -15076,15 +15073,15 @@
       <c r="A27" s="181" t="s">
         <v>489</v>
       </c>
-      <c r="B27" s="393"/>
+      <c r="B27" s="388"/>
       <c r="C27" s="186" t="s">
         <v>438</v>
       </c>
-      <c r="D27" s="382"/>
+      <c r="D27" s="366"/>
       <c r="E27" s="181" t="s">
         <v>522</v>
       </c>
-      <c r="F27" s="393"/>
+      <c r="F27" s="388"/>
       <c r="G27" s="171"/>
       <c r="H27" s="169"/>
       <c r="I27" s="175"/>
@@ -15096,13 +15093,13 @@
       <c r="A28" s="181" t="s">
         <v>490</v>
       </c>
-      <c r="B28" s="393" t="s">
+      <c r="B28" s="388" t="s">
         <v>411</v>
       </c>
       <c r="C28" s="186" t="s">
         <v>439</v>
       </c>
-      <c r="D28" s="382" t="s">
+      <c r="D28" s="366" t="s">
         <v>461</v>
       </c>
       <c r="E28" s="181" t="s">
@@ -15122,11 +15119,11 @@
       <c r="A29" s="181" t="s">
         <v>491</v>
       </c>
-      <c r="B29" s="393"/>
+      <c r="B29" s="388"/>
       <c r="C29" s="186" t="s">
         <v>440</v>
       </c>
-      <c r="D29" s="382"/>
+      <c r="D29" s="366"/>
       <c r="E29" s="181" t="s">
         <v>507</v>
       </c>
@@ -15144,13 +15141,13 @@
       <c r="A30" s="181" t="s">
         <v>492</v>
       </c>
-      <c r="B30" s="393" t="s">
+      <c r="B30" s="388" t="s">
         <v>412</v>
       </c>
       <c r="C30" s="186" t="s">
         <v>441</v>
       </c>
-      <c r="D30" s="382" t="s">
+      <c r="D30" s="366" t="s">
         <v>462</v>
       </c>
       <c r="E30" s="181" t="s">
@@ -15170,11 +15167,11 @@
       <c r="A31" s="181" t="s">
         <v>493</v>
       </c>
-      <c r="B31" s="393"/>
+      <c r="B31" s="388"/>
       <c r="C31" s="186" t="s">
         <v>442</v>
       </c>
-      <c r="D31" s="382"/>
+      <c r="D31" s="366"/>
       <c r="E31" s="181" t="s">
         <v>509</v>
       </c>
@@ -15192,13 +15189,13 @@
       <c r="A32" s="181" t="s">
         <v>494</v>
       </c>
-      <c r="B32" s="393" t="s">
+      <c r="B32" s="388" t="s">
         <v>413</v>
       </c>
       <c r="C32" s="186" t="s">
         <v>443</v>
       </c>
-      <c r="D32" s="382" t="s">
+      <c r="D32" s="366" t="s">
         <v>463</v>
       </c>
       <c r="E32" s="181" t="s">
@@ -15218,11 +15215,11 @@
       <c r="A33" s="181" t="s">
         <v>495</v>
       </c>
-      <c r="B33" s="393"/>
+      <c r="B33" s="388"/>
       <c r="C33" s="186" t="s">
         <v>444</v>
       </c>
-      <c r="D33" s="382"/>
+      <c r="D33" s="366"/>
       <c r="E33" s="181" t="s">
         <v>511</v>
       </c>
@@ -15240,13 +15237,13 @@
       <c r="A34" s="181" t="s">
         <v>496</v>
       </c>
-      <c r="B34" s="393" t="s">
+      <c r="B34" s="388" t="s">
         <v>414</v>
       </c>
       <c r="C34" s="186" t="s">
         <v>445</v>
       </c>
-      <c r="D34" s="382" t="s">
+      <c r="D34" s="366" t="s">
         <v>464</v>
       </c>
       <c r="E34" s="181" t="s">
@@ -15266,11 +15263,11 @@
       <c r="A35" s="182" t="s">
         <v>497</v>
       </c>
-      <c r="B35" s="394"/>
+      <c r="B35" s="389"/>
       <c r="C35" s="187" t="s">
         <v>446</v>
       </c>
-      <c r="D35" s="391"/>
+      <c r="D35" s="367"/>
       <c r="E35" s="182" t="s">
         <v>513</v>
       </c>
@@ -15286,6 +15283,55 @@
     </row>
   </sheetData>
   <mergeCells count="65">
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="H18:H19"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="K9:L9"/>
     <mergeCell ref="L10:L11"/>
@@ -15302,55 +15348,6 @@
     <mergeCell ref="H4:H5"/>
     <mergeCell ref="H6:H7"/>
     <mergeCell ref="H8:H9"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="F22:F23"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="B22:B23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>